<commit_message>
Deploy Appium E2E & Backend reports for build 8
</commit_message>
<xml_diff>
--- a/reports/latest/Backend_Test_Report.xlsx
+++ b/reports/latest/Backend_Test_Report.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22 09:03:12</t>
+          <t>2026-06-22 09:03:28</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -855,7 +855,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -919,7 +919,7 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,7 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1495,7 +1495,7 @@
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1655,7 @@
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1719,7 @@
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -1975,7 +1975,7 @@
       </c>
       <c r="F43" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2039,7 +2039,7 @@
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2167,7 @@
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2295,7 +2295,7 @@
       </c>
       <c r="F53" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2487,7 +2487,7 @@
       </c>
       <c r="F59" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2519,7 +2519,7 @@
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2647,7 @@
       </c>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2679,7 @@
       </c>
       <c r="F65" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2775,7 @@
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2807,7 +2807,7 @@
       </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="F70" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="F71" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="F72" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="F73" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="F74" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="F75" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3063,7 @@
       </c>
       <c r="F77" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="F78" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3127,7 @@
       </c>
       <c r="F79" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3159,7 +3159,7 @@
       </c>
       <c r="F80" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="F81" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="F83" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="F84" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3319,7 @@
       </c>
       <c r="F85" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="F86" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="F87" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3415,7 +3415,7 @@
       </c>
       <c r="F88" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3447,7 +3447,7 @@
       </c>
       <c r="F89" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="F90" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="F91" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3543,7 +3543,7 @@
       </c>
       <c r="F92" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="F93" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3607,7 +3607,7 @@
       </c>
       <c r="F94" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3639,7 +3639,7 @@
       </c>
       <c r="F95" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="F96" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3703,7 +3703,7 @@
       </c>
       <c r="F97" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3735,7 +3735,7 @@
       </c>
       <c r="F98" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="F99" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="F100" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="F101" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="F102" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="F103" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="F104" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3959,7 +3959,7 @@
       </c>
       <c r="F105" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="F106" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="F107" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4055,7 @@
       </c>
       <c r="F108" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4087,7 +4087,7 @@
       </c>
       <c r="F109" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4119,7 +4119,7 @@
       </c>
       <c r="F110" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="F111" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="F112" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4215,7 +4215,7 @@
       </c>
       <c r="F113" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="F114" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4279,7 +4279,7 @@
       </c>
       <c r="F115" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4311,7 +4311,7 @@
       </c>
       <c r="F116" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="F117" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
       </c>
       <c r="F118" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="F119" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4439,7 +4439,7 @@
       </c>
       <c r="F120" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="F121" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4503,7 +4503,7 @@
       </c>
       <c r="F122" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
       </c>
       <c r="F123" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="F124" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4599,7 +4599,7 @@
       </c>
       <c r="F125" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="F126" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4663,7 +4663,7 @@
       </c>
       <c r="F127" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4695,7 +4695,7 @@
       </c>
       <c r="F128" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="F129" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="F130" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4791,7 +4791,7 @@
       </c>
       <c r="F131" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="F132" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4855,7 +4855,7 @@
       </c>
       <c r="F133" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4887,7 +4887,7 @@
       </c>
       <c r="F134" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="F135" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4951,7 +4951,7 @@
       </c>
       <c r="F136" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="F137" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5015,7 +5015,7 @@
       </c>
       <c r="F138" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5047,7 +5047,7 @@
       </c>
       <c r="F139" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="F140" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5111,7 @@
       </c>
       <c r="F141" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5143,7 +5143,7 @@
       </c>
       <c r="F142" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="F143" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5207,7 +5207,7 @@
       </c>
       <c r="F144" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="F145" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
       </c>
       <c r="F146" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5303,7 +5303,7 @@
       </c>
       <c r="F147" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="F148" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5367,7 +5367,7 @@
       </c>
       <c r="F149" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5399,7 +5399,7 @@
       </c>
       <c r="F150" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5431,7 +5431,7 @@
       </c>
       <c r="F151" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5463,7 +5463,7 @@
       </c>
       <c r="F152" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5495,7 +5495,7 @@
       </c>
       <c r="F153" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5527,7 +5527,7 @@
       </c>
       <c r="F154" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5559,7 +5559,7 @@
       </c>
       <c r="F155" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5591,7 +5591,7 @@
       </c>
       <c r="F156" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5623,7 +5623,7 @@
       </c>
       <c r="F157" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5655,7 +5655,7 @@
       </c>
       <c r="F158" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5687,7 +5687,7 @@
       </c>
       <c r="F159" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5719,7 +5719,7 @@
       </c>
       <c r="F160" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5751,7 +5751,7 @@
       </c>
       <c r="F161" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5783,7 +5783,7 @@
       </c>
       <c r="F162" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5815,7 +5815,7 @@
       </c>
       <c r="F163" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="F164" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5879,7 +5879,7 @@
       </c>
       <c r="F165" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5911,7 +5911,7 @@
       </c>
       <c r="F166" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5943,7 +5943,7 @@
       </c>
       <c r="F167" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -5975,7 +5975,7 @@
       </c>
       <c r="F168" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6007,7 +6007,7 @@
       </c>
       <c r="F169" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6039,7 +6039,7 @@
       </c>
       <c r="F170" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6071,7 +6071,7 @@
       </c>
       <c r="F171" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6103,7 +6103,7 @@
       </c>
       <c r="F172" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6135,7 +6135,7 @@
       </c>
       <c r="F173" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6167,7 +6167,7 @@
       </c>
       <c r="F174" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6199,7 +6199,7 @@
       </c>
       <c r="F175" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6231,7 +6231,7 @@
       </c>
       <c r="F176" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6263,7 +6263,7 @@
       </c>
       <c r="F177" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6295,7 +6295,7 @@
       </c>
       <c r="F178" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6327,7 +6327,7 @@
       </c>
       <c r="F179" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6359,7 +6359,7 @@
       </c>
       <c r="F180" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="F181" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6423,7 +6423,7 @@
       </c>
       <c r="F182" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6455,7 +6455,7 @@
       </c>
       <c r="F183" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6487,7 +6487,7 @@
       </c>
       <c r="F184" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="F185" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="F186" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6583,7 +6583,7 @@
       </c>
       <c r="F187" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6615,7 +6615,7 @@
       </c>
       <c r="F188" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6647,7 +6647,7 @@
       </c>
       <c r="F189" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6679,7 +6679,7 @@
       </c>
       <c r="F190" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6711,7 +6711,7 @@
       </c>
       <c r="F191" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="F192" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6775,7 +6775,7 @@
       </c>
       <c r="F193" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6807,7 +6807,7 @@
       </c>
       <c r="F194" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6839,7 +6839,7 @@
       </c>
       <c r="F195" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6871,7 +6871,7 @@
       </c>
       <c r="F196" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6903,7 +6903,7 @@
       </c>
       <c r="F197" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6935,7 +6935,7 @@
       </c>
       <c r="F198" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6967,7 +6967,7 @@
       </c>
       <c r="F199" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -6999,7 +6999,7 @@
       </c>
       <c r="F200" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7031,7 +7031,7 @@
       </c>
       <c r="F201" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7063,7 +7063,7 @@
       </c>
       <c r="F202" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7095,7 +7095,7 @@
       </c>
       <c r="F203" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7127,7 +7127,7 @@
       </c>
       <c r="F204" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7159,7 +7159,7 @@
       </c>
       <c r="F205" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7191,7 +7191,7 @@
       </c>
       <c r="F206" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7223,7 +7223,7 @@
       </c>
       <c r="F207" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7255,7 +7255,7 @@
       </c>
       <c r="F208" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7287,7 +7287,7 @@
       </c>
       <c r="F209" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="F210" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7351,7 +7351,7 @@
       </c>
       <c r="F211" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7383,7 +7383,7 @@
       </c>
       <c r="F212" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7415,7 +7415,7 @@
       </c>
       <c r="F213" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7447,7 +7447,7 @@
       </c>
       <c r="F214" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7479,7 +7479,7 @@
       </c>
       <c r="F215" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7511,7 +7511,7 @@
       </c>
       <c r="F216" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7543,7 +7543,7 @@
       </c>
       <c r="F217" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7575,7 +7575,7 @@
       </c>
       <c r="F218" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7607,7 +7607,7 @@
       </c>
       <c r="F219" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7639,7 +7639,7 @@
       </c>
       <c r="F220" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7671,7 +7671,7 @@
       </c>
       <c r="F221" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7703,7 +7703,7 @@
       </c>
       <c r="F222" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7735,7 +7735,7 @@
       </c>
       <c r="F223" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7767,7 +7767,7 @@
       </c>
       <c r="F224" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7799,7 +7799,7 @@
       </c>
       <c r="F225" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7831,7 +7831,7 @@
       </c>
       <c r="F226" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7863,7 +7863,7 @@
       </c>
       <c r="F227" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7895,7 +7895,7 @@
       </c>
       <c r="F228" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7927,7 +7927,7 @@
       </c>
       <c r="F229" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7959,7 +7959,7 @@
       </c>
       <c r="F230" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -7991,7 +7991,7 @@
       </c>
       <c r="F231" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8023,7 +8023,7 @@
       </c>
       <c r="F232" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8055,7 +8055,7 @@
       </c>
       <c r="F233" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8087,7 +8087,7 @@
       </c>
       <c r="F234" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8119,7 +8119,7 @@
       </c>
       <c r="F235" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8151,7 +8151,7 @@
       </c>
       <c r="F236" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8183,7 +8183,7 @@
       </c>
       <c r="F237" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8215,7 +8215,7 @@
       </c>
       <c r="F238" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8247,7 +8247,7 @@
       </c>
       <c r="F239" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8279,7 +8279,7 @@
       </c>
       <c r="F240" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8311,7 +8311,7 @@
       </c>
       <c r="F241" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8343,7 +8343,7 @@
       </c>
       <c r="F242" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8375,7 +8375,7 @@
       </c>
       <c r="F243" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8407,7 +8407,7 @@
       </c>
       <c r="F244" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8439,7 +8439,7 @@
       </c>
       <c r="F245" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8471,7 +8471,7 @@
       </c>
       <c r="F246" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8503,7 +8503,7 @@
       </c>
       <c r="F247" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8535,7 +8535,7 @@
       </c>
       <c r="F248" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8567,7 +8567,7 @@
       </c>
       <c r="F249" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8599,7 +8599,7 @@
       </c>
       <c r="F250" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8631,7 +8631,7 @@
       </c>
       <c r="F251" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8663,7 +8663,7 @@
       </c>
       <c r="F252" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8695,7 +8695,7 @@
       </c>
       <c r="F253" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8727,7 +8727,7 @@
       </c>
       <c r="F254" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8759,7 +8759,7 @@
       </c>
       <c r="F255" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8791,7 +8791,7 @@
       </c>
       <c r="F256" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8823,7 +8823,7 @@
       </c>
       <c r="F257" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8855,7 +8855,7 @@
       </c>
       <c r="F258" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8887,7 +8887,7 @@
       </c>
       <c r="F259" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8919,7 +8919,7 @@
       </c>
       <c r="F260" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8951,7 +8951,7 @@
       </c>
       <c r="F261" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -8983,7 +8983,7 @@
       </c>
       <c r="F262" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9015,7 +9015,7 @@
       </c>
       <c r="F263" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9047,7 +9047,7 @@
       </c>
       <c r="F264" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9079,7 +9079,7 @@
       </c>
       <c r="F265" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9111,7 +9111,7 @@
       </c>
       <c r="F266" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9143,7 +9143,7 @@
       </c>
       <c r="F267" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9175,7 +9175,7 @@
       </c>
       <c r="F268" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9207,7 +9207,7 @@
       </c>
       <c r="F269" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9239,7 +9239,7 @@
       </c>
       <c r="F270" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9271,7 +9271,7 @@
       </c>
       <c r="F271" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9303,7 +9303,7 @@
       </c>
       <c r="F272" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9335,7 +9335,7 @@
       </c>
       <c r="F273" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9367,7 +9367,7 @@
       </c>
       <c r="F274" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9399,7 +9399,7 @@
       </c>
       <c r="F275" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9431,7 +9431,7 @@
       </c>
       <c r="F276" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9463,7 +9463,7 @@
       </c>
       <c r="F277" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9495,7 +9495,7 @@
       </c>
       <c r="F278" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9527,7 +9527,7 @@
       </c>
       <c r="F279" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9559,7 +9559,7 @@
       </c>
       <c r="F280" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9591,7 +9591,7 @@
       </c>
       <c r="F281" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9623,7 +9623,7 @@
       </c>
       <c r="F282" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9655,7 +9655,7 @@
       </c>
       <c r="F283" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9687,7 +9687,7 @@
       </c>
       <c r="F284" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9719,7 +9719,7 @@
       </c>
       <c r="F285" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9751,7 +9751,7 @@
       </c>
       <c r="F286" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9783,7 +9783,7 @@
       </c>
       <c r="F287" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9815,7 +9815,7 @@
       </c>
       <c r="F288" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9847,7 +9847,7 @@
       </c>
       <c r="F289" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9879,7 +9879,7 @@
       </c>
       <c r="F290" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9911,7 +9911,7 @@
       </c>
       <c r="F291" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9943,7 +9943,7 @@
       </c>
       <c r="F292" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -9975,7 +9975,7 @@
       </c>
       <c r="F293" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -10007,7 +10007,7 @@
       </c>
       <c r="F294" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -10039,7 +10039,7 @@
       </c>
       <c r="F295" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -10071,7 +10071,7 @@
       </c>
       <c r="F296" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -10103,7 +10103,7 @@
       </c>
       <c r="F297" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -10135,7 +10135,7 @@
       </c>
       <c r="F298" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -10167,7 +10167,7 @@
       </c>
       <c r="F299" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -10199,7 +10199,7 @@
       </c>
       <c r="F300" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -10231,7 +10231,7 @@
       </c>
       <c r="F301" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -10263,7 +10263,7 @@
       </c>
       <c r="F302" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -10295,7 +10295,7 @@
       </c>
       <c r="F303" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -10327,7 +10327,7 @@
       </c>
       <c r="F304" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>
@@ -10359,7 +10359,7 @@
       </c>
       <c r="F305" s="8" t="inlineStr">
         <is>
-          <t>09:03:12</t>
+          <t>09:03:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploy Appium E2E & Backend reports for build 9
</commit_message>
<xml_diff>
--- a/reports/latest/Backend_Test_Report.xlsx
+++ b/reports/latest/Backend_Test_Report.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22 09:19:07</t>
+          <t>2026-06-22 09:19:21</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -855,7 +855,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -919,7 +919,7 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,7 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1495,7 +1495,7 @@
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1655,7 @@
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1719,7 @@
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -1975,7 +1975,7 @@
       </c>
       <c r="F43" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2039,7 +2039,7 @@
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2167,7 @@
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2295,7 +2295,7 @@
       </c>
       <c r="F53" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2487,7 +2487,7 @@
       </c>
       <c r="F59" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2519,7 +2519,7 @@
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2647,7 @@
       </c>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2679,7 @@
       </c>
       <c r="F65" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2775,7 @@
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2807,7 +2807,7 @@
       </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="F70" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="F71" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="F72" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="F73" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="F74" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="F75" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3063,7 @@
       </c>
       <c r="F77" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="F78" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3127,7 @@
       </c>
       <c r="F79" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3159,7 +3159,7 @@
       </c>
       <c r="F80" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="F81" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="F83" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="F84" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3319,7 @@
       </c>
       <c r="F85" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="F86" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="F87" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3415,7 +3415,7 @@
       </c>
       <c r="F88" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3447,7 +3447,7 @@
       </c>
       <c r="F89" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="F90" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="F91" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3543,7 +3543,7 @@
       </c>
       <c r="F92" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="F93" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3607,7 +3607,7 @@
       </c>
       <c r="F94" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3639,7 +3639,7 @@
       </c>
       <c r="F95" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="F96" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3703,7 +3703,7 @@
       </c>
       <c r="F97" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3735,7 +3735,7 @@
       </c>
       <c r="F98" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="F99" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="F100" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="F101" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="F102" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="F103" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="F104" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3959,7 +3959,7 @@
       </c>
       <c r="F105" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="F106" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="F107" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4055,7 @@
       </c>
       <c r="F108" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4087,7 +4087,7 @@
       </c>
       <c r="F109" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4119,7 +4119,7 @@
       </c>
       <c r="F110" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="F111" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="F112" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4215,7 +4215,7 @@
       </c>
       <c r="F113" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="F114" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4279,7 +4279,7 @@
       </c>
       <c r="F115" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4311,7 +4311,7 @@
       </c>
       <c r="F116" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="F117" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
       </c>
       <c r="F118" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="F119" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4439,7 +4439,7 @@
       </c>
       <c r="F120" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="F121" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4503,7 +4503,7 @@
       </c>
       <c r="F122" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
       </c>
       <c r="F123" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="F124" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4599,7 +4599,7 @@
       </c>
       <c r="F125" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="F126" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4663,7 +4663,7 @@
       </c>
       <c r="F127" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4695,7 +4695,7 @@
       </c>
       <c r="F128" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="F129" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="F130" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4791,7 +4791,7 @@
       </c>
       <c r="F131" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="F132" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4855,7 +4855,7 @@
       </c>
       <c r="F133" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4887,7 +4887,7 @@
       </c>
       <c r="F134" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="F135" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4951,7 +4951,7 @@
       </c>
       <c r="F136" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="F137" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5015,7 +5015,7 @@
       </c>
       <c r="F138" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5047,7 +5047,7 @@
       </c>
       <c r="F139" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="F140" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5111,7 @@
       </c>
       <c r="F141" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5143,7 +5143,7 @@
       </c>
       <c r="F142" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="F143" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5207,7 +5207,7 @@
       </c>
       <c r="F144" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="F145" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
       </c>
       <c r="F146" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5303,7 +5303,7 @@
       </c>
       <c r="F147" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="F148" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5367,7 +5367,7 @@
       </c>
       <c r="F149" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5399,7 +5399,7 @@
       </c>
       <c r="F150" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5431,7 +5431,7 @@
       </c>
       <c r="F151" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5463,7 +5463,7 @@
       </c>
       <c r="F152" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5495,7 +5495,7 @@
       </c>
       <c r="F153" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5527,7 +5527,7 @@
       </c>
       <c r="F154" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5559,7 +5559,7 @@
       </c>
       <c r="F155" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5591,7 +5591,7 @@
       </c>
       <c r="F156" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5623,7 +5623,7 @@
       </c>
       <c r="F157" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5655,7 +5655,7 @@
       </c>
       <c r="F158" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5687,7 +5687,7 @@
       </c>
       <c r="F159" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5719,7 +5719,7 @@
       </c>
       <c r="F160" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5751,7 +5751,7 @@
       </c>
       <c r="F161" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5783,7 +5783,7 @@
       </c>
       <c r="F162" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5815,7 +5815,7 @@
       </c>
       <c r="F163" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="F164" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5879,7 +5879,7 @@
       </c>
       <c r="F165" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5911,7 +5911,7 @@
       </c>
       <c r="F166" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5943,7 +5943,7 @@
       </c>
       <c r="F167" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -5975,7 +5975,7 @@
       </c>
       <c r="F168" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6007,7 +6007,7 @@
       </c>
       <c r="F169" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6039,7 +6039,7 @@
       </c>
       <c r="F170" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6071,7 +6071,7 @@
       </c>
       <c r="F171" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6103,7 +6103,7 @@
       </c>
       <c r="F172" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6135,7 +6135,7 @@
       </c>
       <c r="F173" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6167,7 +6167,7 @@
       </c>
       <c r="F174" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6199,7 +6199,7 @@
       </c>
       <c r="F175" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6231,7 +6231,7 @@
       </c>
       <c r="F176" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6263,7 +6263,7 @@
       </c>
       <c r="F177" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6295,7 +6295,7 @@
       </c>
       <c r="F178" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6327,7 +6327,7 @@
       </c>
       <c r="F179" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6359,7 +6359,7 @@
       </c>
       <c r="F180" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="F181" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6423,7 +6423,7 @@
       </c>
       <c r="F182" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6455,7 +6455,7 @@
       </c>
       <c r="F183" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6487,7 +6487,7 @@
       </c>
       <c r="F184" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="F185" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="F186" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6583,7 +6583,7 @@
       </c>
       <c r="F187" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6615,7 +6615,7 @@
       </c>
       <c r="F188" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6647,7 +6647,7 @@
       </c>
       <c r="F189" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6679,7 +6679,7 @@
       </c>
       <c r="F190" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6711,7 +6711,7 @@
       </c>
       <c r="F191" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="F192" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6775,7 +6775,7 @@
       </c>
       <c r="F193" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6807,7 +6807,7 @@
       </c>
       <c r="F194" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6839,7 +6839,7 @@
       </c>
       <c r="F195" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6871,7 +6871,7 @@
       </c>
       <c r="F196" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6903,7 +6903,7 @@
       </c>
       <c r="F197" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6935,7 +6935,7 @@
       </c>
       <c r="F198" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6967,7 +6967,7 @@
       </c>
       <c r="F199" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -6999,7 +6999,7 @@
       </c>
       <c r="F200" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7031,7 +7031,7 @@
       </c>
       <c r="F201" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7063,7 +7063,7 @@
       </c>
       <c r="F202" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7095,7 +7095,7 @@
       </c>
       <c r="F203" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7127,7 +7127,7 @@
       </c>
       <c r="F204" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7159,7 +7159,7 @@
       </c>
       <c r="F205" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7191,7 +7191,7 @@
       </c>
       <c r="F206" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7223,7 +7223,7 @@
       </c>
       <c r="F207" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7255,7 +7255,7 @@
       </c>
       <c r="F208" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7287,7 +7287,7 @@
       </c>
       <c r="F209" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="F210" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7351,7 +7351,7 @@
       </c>
       <c r="F211" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7383,7 +7383,7 @@
       </c>
       <c r="F212" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7415,7 +7415,7 @@
       </c>
       <c r="F213" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7447,7 +7447,7 @@
       </c>
       <c r="F214" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7479,7 +7479,7 @@
       </c>
       <c r="F215" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7511,7 +7511,7 @@
       </c>
       <c r="F216" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7543,7 +7543,7 @@
       </c>
       <c r="F217" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7575,7 +7575,7 @@
       </c>
       <c r="F218" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7607,7 +7607,7 @@
       </c>
       <c r="F219" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7639,7 +7639,7 @@
       </c>
       <c r="F220" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7671,7 +7671,7 @@
       </c>
       <c r="F221" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7703,7 +7703,7 @@
       </c>
       <c r="F222" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7735,7 +7735,7 @@
       </c>
       <c r="F223" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7767,7 +7767,7 @@
       </c>
       <c r="F224" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7799,7 +7799,7 @@
       </c>
       <c r="F225" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7831,7 +7831,7 @@
       </c>
       <c r="F226" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7863,7 +7863,7 @@
       </c>
       <c r="F227" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7895,7 +7895,7 @@
       </c>
       <c r="F228" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7927,7 +7927,7 @@
       </c>
       <c r="F229" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7959,7 +7959,7 @@
       </c>
       <c r="F230" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -7991,7 +7991,7 @@
       </c>
       <c r="F231" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8023,7 +8023,7 @@
       </c>
       <c r="F232" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8055,7 +8055,7 @@
       </c>
       <c r="F233" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8087,7 +8087,7 @@
       </c>
       <c r="F234" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8119,7 +8119,7 @@
       </c>
       <c r="F235" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8151,7 +8151,7 @@
       </c>
       <c r="F236" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8183,7 +8183,7 @@
       </c>
       <c r="F237" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8215,7 +8215,7 @@
       </c>
       <c r="F238" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8247,7 +8247,7 @@
       </c>
       <c r="F239" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8279,7 +8279,7 @@
       </c>
       <c r="F240" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8311,7 +8311,7 @@
       </c>
       <c r="F241" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8343,7 +8343,7 @@
       </c>
       <c r="F242" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8375,7 +8375,7 @@
       </c>
       <c r="F243" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8407,7 +8407,7 @@
       </c>
       <c r="F244" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8439,7 +8439,7 @@
       </c>
       <c r="F245" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8471,7 +8471,7 @@
       </c>
       <c r="F246" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8503,7 +8503,7 @@
       </c>
       <c r="F247" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8535,7 +8535,7 @@
       </c>
       <c r="F248" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8567,7 +8567,7 @@
       </c>
       <c r="F249" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8599,7 +8599,7 @@
       </c>
       <c r="F250" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8631,7 +8631,7 @@
       </c>
       <c r="F251" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8663,7 +8663,7 @@
       </c>
       <c r="F252" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8695,7 +8695,7 @@
       </c>
       <c r="F253" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8727,7 +8727,7 @@
       </c>
       <c r="F254" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8759,7 +8759,7 @@
       </c>
       <c r="F255" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8791,7 +8791,7 @@
       </c>
       <c r="F256" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8823,7 +8823,7 @@
       </c>
       <c r="F257" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8855,7 +8855,7 @@
       </c>
       <c r="F258" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8887,7 +8887,7 @@
       </c>
       <c r="F259" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8919,7 +8919,7 @@
       </c>
       <c r="F260" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8951,7 +8951,7 @@
       </c>
       <c r="F261" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -8983,7 +8983,7 @@
       </c>
       <c r="F262" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9015,7 +9015,7 @@
       </c>
       <c r="F263" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9047,7 +9047,7 @@
       </c>
       <c r="F264" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9079,7 +9079,7 @@
       </c>
       <c r="F265" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9111,7 +9111,7 @@
       </c>
       <c r="F266" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9143,7 +9143,7 @@
       </c>
       <c r="F267" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9175,7 +9175,7 @@
       </c>
       <c r="F268" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9207,7 +9207,7 @@
       </c>
       <c r="F269" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9239,7 +9239,7 @@
       </c>
       <c r="F270" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9271,7 +9271,7 @@
       </c>
       <c r="F271" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9303,7 +9303,7 @@
       </c>
       <c r="F272" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9335,7 +9335,7 @@
       </c>
       <c r="F273" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9367,7 +9367,7 @@
       </c>
       <c r="F274" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9399,7 +9399,7 @@
       </c>
       <c r="F275" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9431,7 +9431,7 @@
       </c>
       <c r="F276" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9463,7 +9463,7 @@
       </c>
       <c r="F277" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9495,7 +9495,7 @@
       </c>
       <c r="F278" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9527,7 +9527,7 @@
       </c>
       <c r="F279" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9559,7 +9559,7 @@
       </c>
       <c r="F280" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9591,7 +9591,7 @@
       </c>
       <c r="F281" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9623,7 +9623,7 @@
       </c>
       <c r="F282" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9655,7 +9655,7 @@
       </c>
       <c r="F283" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9687,7 +9687,7 @@
       </c>
       <c r="F284" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9719,7 +9719,7 @@
       </c>
       <c r="F285" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9751,7 +9751,7 @@
       </c>
       <c r="F286" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9783,7 +9783,7 @@
       </c>
       <c r="F287" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9815,7 +9815,7 @@
       </c>
       <c r="F288" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9847,7 +9847,7 @@
       </c>
       <c r="F289" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9879,7 +9879,7 @@
       </c>
       <c r="F290" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9911,7 +9911,7 @@
       </c>
       <c r="F291" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9943,7 +9943,7 @@
       </c>
       <c r="F292" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -9975,7 +9975,7 @@
       </c>
       <c r="F293" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -10007,7 +10007,7 @@
       </c>
       <c r="F294" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -10039,7 +10039,7 @@
       </c>
       <c r="F295" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -10071,7 +10071,7 @@
       </c>
       <c r="F296" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -10103,7 +10103,7 @@
       </c>
       <c r="F297" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -10135,7 +10135,7 @@
       </c>
       <c r="F298" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -10167,7 +10167,7 @@
       </c>
       <c r="F299" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -10199,7 +10199,7 @@
       </c>
       <c r="F300" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -10231,7 +10231,7 @@
       </c>
       <c r="F301" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -10263,7 +10263,7 @@
       </c>
       <c r="F302" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -10295,7 +10295,7 @@
       </c>
       <c r="F303" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -10327,7 +10327,7 @@
       </c>
       <c r="F304" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>
@@ -10359,7 +10359,7 @@
       </c>
       <c r="F305" s="8" t="inlineStr">
         <is>
-          <t>09:19:07</t>
+          <t>09:19:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploy Appium E2E & Backend reports for build 10
</commit_message>
<xml_diff>
--- a/reports/latest/Backend_Test_Report.xlsx
+++ b/reports/latest/Backend_Test_Report.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22 09:26:12</t>
+          <t>2026-06-22 09:26:19</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -855,7 +855,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -919,7 +919,7 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,7 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1495,7 +1495,7 @@
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1655,7 @@
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1719,7 @@
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -1975,7 +1975,7 @@
       </c>
       <c r="F43" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2039,7 +2039,7 @@
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2167,7 @@
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2295,7 +2295,7 @@
       </c>
       <c r="F53" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2487,7 +2487,7 @@
       </c>
       <c r="F59" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2519,7 +2519,7 @@
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2647,7 @@
       </c>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2679,7 @@
       </c>
       <c r="F65" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2775,7 @@
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2807,7 +2807,7 @@
       </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="F70" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="F71" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="F72" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="F73" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="F74" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="F75" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3063,7 @@
       </c>
       <c r="F77" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="F78" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3127,7 @@
       </c>
       <c r="F79" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3159,7 +3159,7 @@
       </c>
       <c r="F80" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="F81" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="F83" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="F84" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3319,7 @@
       </c>
       <c r="F85" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="F86" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="F87" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3415,7 +3415,7 @@
       </c>
       <c r="F88" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3447,7 +3447,7 @@
       </c>
       <c r="F89" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="F90" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="F91" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3543,7 +3543,7 @@
       </c>
       <c r="F92" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="F93" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3607,7 +3607,7 @@
       </c>
       <c r="F94" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3639,7 +3639,7 @@
       </c>
       <c r="F95" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="F96" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3703,7 +3703,7 @@
       </c>
       <c r="F97" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3735,7 +3735,7 @@
       </c>
       <c r="F98" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="F99" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="F100" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="F101" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="F102" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="F103" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="F104" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3959,7 +3959,7 @@
       </c>
       <c r="F105" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="F106" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="F107" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4055,7 @@
       </c>
       <c r="F108" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4087,7 +4087,7 @@
       </c>
       <c r="F109" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4119,7 +4119,7 @@
       </c>
       <c r="F110" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="F111" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="F112" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4215,7 +4215,7 @@
       </c>
       <c r="F113" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="F114" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4279,7 +4279,7 @@
       </c>
       <c r="F115" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4311,7 +4311,7 @@
       </c>
       <c r="F116" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="F117" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
       </c>
       <c r="F118" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="F119" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4439,7 +4439,7 @@
       </c>
       <c r="F120" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="F121" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4503,7 +4503,7 @@
       </c>
       <c r="F122" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
       </c>
       <c r="F123" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="F124" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4599,7 +4599,7 @@
       </c>
       <c r="F125" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="F126" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4663,7 +4663,7 @@
       </c>
       <c r="F127" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4695,7 +4695,7 @@
       </c>
       <c r="F128" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="F129" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="F130" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4791,7 +4791,7 @@
       </c>
       <c r="F131" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="F132" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4855,7 +4855,7 @@
       </c>
       <c r="F133" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4887,7 +4887,7 @@
       </c>
       <c r="F134" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="F135" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4951,7 +4951,7 @@
       </c>
       <c r="F136" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="F137" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5015,7 +5015,7 @@
       </c>
       <c r="F138" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5047,7 +5047,7 @@
       </c>
       <c r="F139" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="F140" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5111,7 @@
       </c>
       <c r="F141" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5143,7 +5143,7 @@
       </c>
       <c r="F142" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="F143" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5207,7 +5207,7 @@
       </c>
       <c r="F144" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="F145" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
       </c>
       <c r="F146" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5303,7 +5303,7 @@
       </c>
       <c r="F147" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="F148" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5367,7 +5367,7 @@
       </c>
       <c r="F149" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5399,7 +5399,7 @@
       </c>
       <c r="F150" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5431,7 +5431,7 @@
       </c>
       <c r="F151" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5463,7 +5463,7 @@
       </c>
       <c r="F152" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5495,7 +5495,7 @@
       </c>
       <c r="F153" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5527,7 +5527,7 @@
       </c>
       <c r="F154" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5559,7 +5559,7 @@
       </c>
       <c r="F155" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5591,7 +5591,7 @@
       </c>
       <c r="F156" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5623,7 +5623,7 @@
       </c>
       <c r="F157" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5655,7 +5655,7 @@
       </c>
       <c r="F158" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5687,7 +5687,7 @@
       </c>
       <c r="F159" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5719,7 +5719,7 @@
       </c>
       <c r="F160" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5751,7 +5751,7 @@
       </c>
       <c r="F161" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5783,7 +5783,7 @@
       </c>
       <c r="F162" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5815,7 +5815,7 @@
       </c>
       <c r="F163" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="F164" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5879,7 +5879,7 @@
       </c>
       <c r="F165" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5911,7 +5911,7 @@
       </c>
       <c r="F166" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5943,7 +5943,7 @@
       </c>
       <c r="F167" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -5975,7 +5975,7 @@
       </c>
       <c r="F168" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6007,7 +6007,7 @@
       </c>
       <c r="F169" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6039,7 +6039,7 @@
       </c>
       <c r="F170" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6071,7 +6071,7 @@
       </c>
       <c r="F171" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6103,7 +6103,7 @@
       </c>
       <c r="F172" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6135,7 +6135,7 @@
       </c>
       <c r="F173" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6167,7 +6167,7 @@
       </c>
       <c r="F174" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6199,7 +6199,7 @@
       </c>
       <c r="F175" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6231,7 +6231,7 @@
       </c>
       <c r="F176" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6263,7 +6263,7 @@
       </c>
       <c r="F177" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6295,7 +6295,7 @@
       </c>
       <c r="F178" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6327,7 +6327,7 @@
       </c>
       <c r="F179" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6359,7 +6359,7 @@
       </c>
       <c r="F180" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="F181" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6423,7 +6423,7 @@
       </c>
       <c r="F182" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6455,7 +6455,7 @@
       </c>
       <c r="F183" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6487,7 +6487,7 @@
       </c>
       <c r="F184" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="F185" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="F186" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6583,7 +6583,7 @@
       </c>
       <c r="F187" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6615,7 +6615,7 @@
       </c>
       <c r="F188" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6647,7 +6647,7 @@
       </c>
       <c r="F189" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6679,7 +6679,7 @@
       </c>
       <c r="F190" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6711,7 +6711,7 @@
       </c>
       <c r="F191" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="F192" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6775,7 +6775,7 @@
       </c>
       <c r="F193" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6807,7 +6807,7 @@
       </c>
       <c r="F194" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6839,7 +6839,7 @@
       </c>
       <c r="F195" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6871,7 +6871,7 @@
       </c>
       <c r="F196" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6903,7 +6903,7 @@
       </c>
       <c r="F197" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6935,7 +6935,7 @@
       </c>
       <c r="F198" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6967,7 +6967,7 @@
       </c>
       <c r="F199" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -6999,7 +6999,7 @@
       </c>
       <c r="F200" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7031,7 +7031,7 @@
       </c>
       <c r="F201" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7063,7 +7063,7 @@
       </c>
       <c r="F202" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7095,7 +7095,7 @@
       </c>
       <c r="F203" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7127,7 +7127,7 @@
       </c>
       <c r="F204" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7159,7 +7159,7 @@
       </c>
       <c r="F205" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7191,7 +7191,7 @@
       </c>
       <c r="F206" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7223,7 +7223,7 @@
       </c>
       <c r="F207" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7255,7 +7255,7 @@
       </c>
       <c r="F208" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7287,7 +7287,7 @@
       </c>
       <c r="F209" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="F210" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7351,7 +7351,7 @@
       </c>
       <c r="F211" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7383,7 +7383,7 @@
       </c>
       <c r="F212" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7415,7 +7415,7 @@
       </c>
       <c r="F213" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7447,7 +7447,7 @@
       </c>
       <c r="F214" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7479,7 +7479,7 @@
       </c>
       <c r="F215" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7511,7 +7511,7 @@
       </c>
       <c r="F216" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7543,7 +7543,7 @@
       </c>
       <c r="F217" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7575,7 +7575,7 @@
       </c>
       <c r="F218" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7607,7 +7607,7 @@
       </c>
       <c r="F219" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7639,7 +7639,7 @@
       </c>
       <c r="F220" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7671,7 +7671,7 @@
       </c>
       <c r="F221" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7703,7 +7703,7 @@
       </c>
       <c r="F222" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7735,7 +7735,7 @@
       </c>
       <c r="F223" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7767,7 +7767,7 @@
       </c>
       <c r="F224" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7799,7 +7799,7 @@
       </c>
       <c r="F225" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7831,7 +7831,7 @@
       </c>
       <c r="F226" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7863,7 +7863,7 @@
       </c>
       <c r="F227" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7895,7 +7895,7 @@
       </c>
       <c r="F228" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7927,7 +7927,7 @@
       </c>
       <c r="F229" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7959,7 +7959,7 @@
       </c>
       <c r="F230" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -7991,7 +7991,7 @@
       </c>
       <c r="F231" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8023,7 +8023,7 @@
       </c>
       <c r="F232" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8055,7 +8055,7 @@
       </c>
       <c r="F233" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8087,7 +8087,7 @@
       </c>
       <c r="F234" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8119,7 +8119,7 @@
       </c>
       <c r="F235" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8151,7 +8151,7 @@
       </c>
       <c r="F236" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8183,7 +8183,7 @@
       </c>
       <c r="F237" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8215,7 +8215,7 @@
       </c>
       <c r="F238" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8247,7 +8247,7 @@
       </c>
       <c r="F239" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8279,7 +8279,7 @@
       </c>
       <c r="F240" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8311,7 +8311,7 @@
       </c>
       <c r="F241" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8343,7 +8343,7 @@
       </c>
       <c r="F242" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8375,7 +8375,7 @@
       </c>
       <c r="F243" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8407,7 +8407,7 @@
       </c>
       <c r="F244" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8439,7 +8439,7 @@
       </c>
       <c r="F245" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8471,7 +8471,7 @@
       </c>
       <c r="F246" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8503,7 +8503,7 @@
       </c>
       <c r="F247" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8535,7 +8535,7 @@
       </c>
       <c r="F248" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8567,7 +8567,7 @@
       </c>
       <c r="F249" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8599,7 +8599,7 @@
       </c>
       <c r="F250" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8631,7 +8631,7 @@
       </c>
       <c r="F251" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8663,7 +8663,7 @@
       </c>
       <c r="F252" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8695,7 +8695,7 @@
       </c>
       <c r="F253" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8727,7 +8727,7 @@
       </c>
       <c r="F254" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8759,7 +8759,7 @@
       </c>
       <c r="F255" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8791,7 +8791,7 @@
       </c>
       <c r="F256" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8823,7 +8823,7 @@
       </c>
       <c r="F257" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8855,7 +8855,7 @@
       </c>
       <c r="F258" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8887,7 +8887,7 @@
       </c>
       <c r="F259" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8919,7 +8919,7 @@
       </c>
       <c r="F260" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8951,7 +8951,7 @@
       </c>
       <c r="F261" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -8983,7 +8983,7 @@
       </c>
       <c r="F262" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9015,7 +9015,7 @@
       </c>
       <c r="F263" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9047,7 +9047,7 @@
       </c>
       <c r="F264" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9079,7 +9079,7 @@
       </c>
       <c r="F265" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9111,7 +9111,7 @@
       </c>
       <c r="F266" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9143,7 +9143,7 @@
       </c>
       <c r="F267" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9175,7 +9175,7 @@
       </c>
       <c r="F268" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9207,7 +9207,7 @@
       </c>
       <c r="F269" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9239,7 +9239,7 @@
       </c>
       <c r="F270" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9271,7 +9271,7 @@
       </c>
       <c r="F271" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9303,7 +9303,7 @@
       </c>
       <c r="F272" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9335,7 +9335,7 @@
       </c>
       <c r="F273" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9367,7 +9367,7 @@
       </c>
       <c r="F274" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9399,7 +9399,7 @@
       </c>
       <c r="F275" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9431,7 +9431,7 @@
       </c>
       <c r="F276" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9463,7 +9463,7 @@
       </c>
       <c r="F277" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9495,7 +9495,7 @@
       </c>
       <c r="F278" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9527,7 +9527,7 @@
       </c>
       <c r="F279" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9559,7 +9559,7 @@
       </c>
       <c r="F280" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9591,7 +9591,7 @@
       </c>
       <c r="F281" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9623,7 +9623,7 @@
       </c>
       <c r="F282" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9655,7 +9655,7 @@
       </c>
       <c r="F283" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9687,7 +9687,7 @@
       </c>
       <c r="F284" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9719,7 +9719,7 @@
       </c>
       <c r="F285" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9751,7 +9751,7 @@
       </c>
       <c r="F286" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9783,7 +9783,7 @@
       </c>
       <c r="F287" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9815,7 +9815,7 @@
       </c>
       <c r="F288" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9847,7 +9847,7 @@
       </c>
       <c r="F289" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9879,7 +9879,7 @@
       </c>
       <c r="F290" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9911,7 +9911,7 @@
       </c>
       <c r="F291" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9943,7 +9943,7 @@
       </c>
       <c r="F292" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -9975,7 +9975,7 @@
       </c>
       <c r="F293" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -10007,7 +10007,7 @@
       </c>
       <c r="F294" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -10039,7 +10039,7 @@
       </c>
       <c r="F295" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -10071,7 +10071,7 @@
       </c>
       <c r="F296" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -10103,7 +10103,7 @@
       </c>
       <c r="F297" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -10135,7 +10135,7 @@
       </c>
       <c r="F298" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -10167,7 +10167,7 @@
       </c>
       <c r="F299" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -10199,7 +10199,7 @@
       </c>
       <c r="F300" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -10231,7 +10231,7 @@
       </c>
       <c r="F301" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -10263,7 +10263,7 @@
       </c>
       <c r="F302" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -10295,7 +10295,7 @@
       </c>
       <c r="F303" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -10327,7 +10327,7 @@
       </c>
       <c r="F304" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>
@@ -10359,7 +10359,7 @@
       </c>
       <c r="F305" s="8" t="inlineStr">
         <is>
-          <t>09:26:12</t>
+          <t>09:26:19</t>
         </is>
       </c>
     </row>

</xml_diff>